<commit_message>
Spreadsheet update-A10059 & A90050
</commit_message>
<xml_diff>
--- a/data/PPP-2027-Review-Tracking.xlsx
+++ b/data/PPP-2027-Review-Tracking.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ashtd-my.sharepoint.com/personal/niwesh_koirala_ardot_gov/Documents/Desktop/Github/PPP-2027-Review-Control-Center/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="7" documentId="13_ncr:1_{96CAE750-3891-4C13-A1A6-B95BF8A82FAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0D27CFAE-FEC2-4068-84D9-3182921FEB6B}"/>
+  <xr:revisionPtr revIDLastSave="12" documentId="13_ncr:1_{96CAE750-3891-4C13-A1A6-B95BF8A82FAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5195AC65-1A6A-41C0-AF53-30BF82D7C28C}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="675" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1505,8 +1505,12 @@
       <c r="P2" s="20">
         <v>46262</v>
       </c>
-      <c r="Q2" s="20"/>
-      <c r="R2" s="20"/>
+      <c r="Q2" s="20">
+        <v>46266</v>
+      </c>
+      <c r="R2" s="20">
+        <v>46266</v>
+      </c>
       <c r="S2" s="20"/>
       <c r="T2" s="20"/>
       <c r="U2" s="20"/>
@@ -1639,7 +1643,7 @@
         <v>46266</v>
       </c>
       <c r="V4" s="20">
-        <v>46267</v>
+        <v>46266</v>
       </c>
       <c r="W4" s="20"/>
       <c r="X4" s="20"/>
@@ -2086,8 +2090,12 @@
       <c r="T12" s="20">
         <v>46248</v>
       </c>
-      <c r="U12" s="20"/>
-      <c r="V12" s="20"/>
+      <c r="U12" s="20">
+        <v>46266</v>
+      </c>
+      <c r="V12" s="20">
+        <v>46266</v>
+      </c>
       <c r="W12" s="20"/>
       <c r="X12" s="20"/>
       <c r="AK12" s="24" t="s">

</xml_diff>

<commit_message>
Spreadsheet update-A90051 & A60066
</commit_message>
<xml_diff>
--- a/data/PPP-2027-Review-Tracking.xlsx
+++ b/data/PPP-2027-Review-Tracking.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ashtd-my.sharepoint.com/personal/niwesh_koirala_ardot_gov/Documents/Desktop/Github/PPP-2027-Review-Control-Center/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="12" documentId="13_ncr:1_{96CAE750-3891-4C13-A1A6-B95BF8A82FAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5195AC65-1A6A-41C0-AF53-30BF82D7C28C}"/>
+  <xr:revisionPtr revIDLastSave="15" documentId="13_ncr:1_{96CAE750-3891-4C13-A1A6-B95BF8A82FAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{33631FF9-7269-4833-8A43-E6FF0B6D526C}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="675" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1849,8 +1849,12 @@
       <c r="N8" s="20">
         <v>46265</v>
       </c>
-      <c r="O8" s="20"/>
-      <c r="P8" s="20"/>
+      <c r="O8" s="20">
+        <v>46266</v>
+      </c>
+      <c r="P8" s="20">
+        <v>46266</v>
+      </c>
       <c r="Q8" s="20"/>
       <c r="R8" s="20"/>
       <c r="S8" s="20"/>
@@ -2174,6 +2178,9 @@
       </c>
       <c r="X13" s="20">
         <v>46265</v>
+      </c>
+      <c r="Y13" s="20">
+        <v>46266</v>
       </c>
     </row>
     <row r="14" spans="1:37">

</xml_diff>

<commit_message>
Spreadsheet update-AX0012 & A10058
</commit_message>
<xml_diff>
--- a/data/PPP-2027-Review-Tracking.xlsx
+++ b/data/PPP-2027-Review-Tracking.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ashtd-my.sharepoint.com/personal/niwesh_koirala_ardot_gov/Documents/Desktop/Github/PPP-2027-Review-Control-Center/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="26" documentId="13_ncr:1_{96CAE750-3891-4C13-A1A6-B95BF8A82FAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{24C392DB-EDAC-46F2-BD4E-9117F7796177}"/>
+  <xr:revisionPtr revIDLastSave="29" documentId="13_ncr:1_{96CAE750-3891-4C13-A1A6-B95BF8A82FAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{73B5ED7F-EB4F-4607-85A4-6D4CA26AACB9}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="675" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -786,7 +786,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -829,8 +829,20 @@
       <name val="Segoe UI"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Arial Narrow"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="14">
+  <fills count="15">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -897,8 +909,13 @@
         <fgColor rgb="FFF2EAFE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -935,12 +952,28 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1001,8 +1034,12 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="14" fontId="8" fillId="0" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
+    <cellStyle name="Good" xfId="2" builtinId="26"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{2A31118A-900B-4722-A90B-8152F5F4035D}"/>
   </cellStyles>
@@ -2287,8 +2324,12 @@
       <c r="L15" s="20">
         <v>46259</v>
       </c>
-      <c r="M15" s="20"/>
-      <c r="N15" s="20"/>
+      <c r="M15" s="20">
+        <v>46266</v>
+      </c>
+      <c r="N15" s="20">
+        <v>46267</v>
+      </c>
       <c r="O15" s="20"/>
       <c r="P15" s="20"/>
       <c r="Q15" s="20"/>
@@ -3051,7 +3092,9 @@
       <c r="I33" s="21">
         <v>46363</v>
       </c>
-      <c r="J33" s="21"/>
+      <c r="J33" s="26">
+        <v>46267</v>
+      </c>
       <c r="K33" s="20"/>
       <c r="L33" s="20"/>
       <c r="M33" s="20"/>

</xml_diff>

<commit_message>
Spreadsheet update-A40062 on reminder to District
</commit_message>
<xml_diff>
--- a/data/PPP-2027-Review-Tracking.xlsx
+++ b/data/PPP-2027-Review-Tracking.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ashtd-my.sharepoint.com/personal/niwesh_koirala_ardot_gov/Documents/Desktop/Github/PPP-2027-Review-Control-Center/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="31" documentId="13_ncr:1_{96CAE750-3891-4C13-A1A6-B95BF8A82FAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{64BF21E9-A233-49D9-81E6-335411129C22}"/>
+  <xr:revisionPtr revIDLastSave="33" documentId="13_ncr:1_{96CAE750-3891-4C13-A1A6-B95BF8A82FAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8B35568B-8248-4A04-8ED9-D7177EF8794A}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="675" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="353" uniqueCount="253">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="254">
   <si>
     <t>1st Review</t>
   </si>
@@ -780,6 +780,9 @@
   </si>
   <si>
     <t>Roadway additional comment was send to District on 8.14.2026. Email was send for an update on 8.31.2026</t>
+  </si>
+  <si>
+    <t>Reminder send to District (Marcus for the update) on 9.2.2026</t>
   </si>
 </sst>
 </file>
@@ -1748,6 +1751,9 @@
       <c r="V5" s="20"/>
       <c r="W5" s="20"/>
       <c r="X5" s="20"/>
+      <c r="AK5" s="24" t="s">
+        <v>253</v>
+      </c>
     </row>
     <row r="6" spans="1:37">
       <c r="A6" s="11" t="s">

</xml_diff>

<commit_message>
Spreadsheet updates-A90050 & A30049
</commit_message>
<xml_diff>
--- a/data/PPP-2027-Review-Tracking.xlsx
+++ b/data/PPP-2027-Review-Tracking.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ashtd-my.sharepoint.com/personal/niwesh_koirala_ardot_gov/Documents/Desktop/Github/PPP-2027-Review-Control-Center/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="33" documentId="13_ncr:1_{96CAE750-3891-4C13-A1A6-B95BF8A82FAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8B35568B-8248-4A04-8ED9-D7177EF8794A}"/>
+  <xr:revisionPtr revIDLastSave="36" documentId="13_ncr:1_{96CAE750-3891-4C13-A1A6-B95BF8A82FAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9D5E816B-A0DB-4EB0-A741-A229ED3AC6E3}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="675" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1699,8 +1699,12 @@
       <c r="V4" s="20">
         <v>46266</v>
       </c>
-      <c r="W4" s="20"/>
-      <c r="X4" s="20"/>
+      <c r="W4" s="20">
+        <v>46267</v>
+      </c>
+      <c r="X4" s="20">
+        <v>46267</v>
+      </c>
     </row>
     <row r="5" spans="1:37">
       <c r="A5" s="11" t="s">
@@ -2157,8 +2161,12 @@
       <c r="V12" s="20">
         <v>46266</v>
       </c>
-      <c r="W12" s="20"/>
-      <c r="X12" s="20"/>
+      <c r="W12" s="20">
+        <v>46267</v>
+      </c>
+      <c r="X12" s="20">
+        <v>46267</v>
+      </c>
       <c r="AK12" s="24" t="s">
         <v>252</v>
       </c>

</xml_diff>

<commit_message>
Spreadsheet updates-In General 9.3.2026
</commit_message>
<xml_diff>
--- a/data/PPP-2027-Review-Tracking.xlsx
+++ b/data/PPP-2027-Review-Tracking.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ashtd-my.sharepoint.com/personal/niwesh_koirala_ardot_gov/Documents/Desktop/Github/PPP-2027-Review-Control-Center/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="36" documentId="13_ncr:1_{96CAE750-3891-4C13-A1A6-B95BF8A82FAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9D5E816B-A0DB-4EB0-A741-A229ED3AC6E3}"/>
+  <xr:revisionPtr revIDLastSave="53" documentId="13_ncr:1_{96CAE750-3891-4C13-A1A6-B95BF8A82FAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DB57B770-2AAD-4F71-94CC-7800840FAA05}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="675" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PPP Projects" sheetId="2" r:id="rId1"/>
@@ -789,7 +789,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -832,20 +832,8 @@
       <name val="Segoe UI"/>
       <family val="2"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Arial Narrow"/>
-      <family val="2"/>
-    </font>
   </fonts>
-  <fills count="15">
+  <fills count="14">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -912,13 +900,8 @@
         <fgColor rgb="FFF2EAFE"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="5">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -955,28 +938,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1037,12 +1004,8 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="14" fontId="8" fillId="0" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
-  <cellStyles count="3">
-    <cellStyle name="Good" xfId="2" builtinId="26"/>
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{2A31118A-900B-4722-A90B-8152F5F4035D}"/>
   </cellStyles>
@@ -1109,6 +1072,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1561,6 +1528,7 @@
       <c r="V2" s="20"/>
       <c r="W2" s="20"/>
       <c r="X2" s="20"/>
+      <c r="Y2" s="20"/>
     </row>
     <row r="3" spans="1:37">
       <c r="A3" s="11" t="s">
@@ -1629,8 +1597,13 @@
       <c r="V3" s="20">
         <v>46267</v>
       </c>
-      <c r="W3" s="20"/>
-      <c r="X3" s="20"/>
+      <c r="W3" s="20">
+        <v>46267</v>
+      </c>
+      <c r="X3" s="20">
+        <v>46267</v>
+      </c>
+      <c r="Y3" s="20"/>
     </row>
     <row r="4" spans="1:37">
       <c r="A4" s="11" t="s">
@@ -1705,6 +1678,7 @@
       <c r="X4" s="20">
         <v>46267</v>
       </c>
+      <c r="Y4" s="20"/>
     </row>
     <row r="5" spans="1:37">
       <c r="A5" s="11" t="s">
@@ -1755,6 +1729,7 @@
       <c r="V5" s="20"/>
       <c r="W5" s="20"/>
       <c r="X5" s="20"/>
+      <c r="Y5" s="20"/>
       <c r="AK5" s="24" t="s">
         <v>253</v>
       </c>
@@ -1816,6 +1791,7 @@
       <c r="V6" s="20"/>
       <c r="W6" s="20"/>
       <c r="X6" s="20"/>
+      <c r="Y6" s="20"/>
     </row>
     <row r="7" spans="1:37">
       <c r="A7" s="11" t="s">
@@ -1866,6 +1842,7 @@
       <c r="V7" s="20"/>
       <c r="W7" s="20"/>
       <c r="X7" s="20"/>
+      <c r="Y7" s="20"/>
     </row>
     <row r="8" spans="1:37">
       <c r="A8" s="11" t="s">
@@ -1924,6 +1901,7 @@
       <c r="V8" s="20"/>
       <c r="W8" s="20"/>
       <c r="X8" s="20"/>
+      <c r="Y8" s="20"/>
       <c r="AK8" s="24" t="s">
         <v>251</v>
       </c>
@@ -1965,10 +1943,18 @@
       <c r="L9" s="25">
         <v>46265</v>
       </c>
-      <c r="M9" s="20"/>
-      <c r="N9" s="20"/>
-      <c r="O9" s="20"/>
-      <c r="P9" s="20"/>
+      <c r="M9" s="20">
+        <v>46266</v>
+      </c>
+      <c r="N9" s="20">
+        <v>46266</v>
+      </c>
+      <c r="O9" s="20">
+        <v>46267</v>
+      </c>
+      <c r="P9" s="20">
+        <v>46268</v>
+      </c>
       <c r="Q9" s="20"/>
       <c r="R9" s="20"/>
       <c r="S9" s="20"/>
@@ -1977,6 +1963,7 @@
       <c r="V9" s="20"/>
       <c r="W9" s="20"/>
       <c r="X9" s="20"/>
+      <c r="Y9" s="20"/>
     </row>
     <row r="10" spans="1:37">
       <c r="A10" s="11" t="s">
@@ -2027,14 +2014,23 @@
       <c r="P10" s="20">
         <v>46265</v>
       </c>
-      <c r="Q10" s="20"/>
-      <c r="R10" s="20"/>
-      <c r="S10" s="20"/>
-      <c r="T10" s="20"/>
+      <c r="Q10" s="20">
+        <v>46267</v>
+      </c>
+      <c r="R10" s="20">
+        <v>46267</v>
+      </c>
+      <c r="S10" s="20">
+        <v>46268</v>
+      </c>
+      <c r="T10" s="20">
+        <v>46268</v>
+      </c>
       <c r="U10" s="20"/>
       <c r="V10" s="20"/>
       <c r="W10" s="20"/>
       <c r="X10" s="20"/>
+      <c r="Y10" s="20"/>
     </row>
     <row r="11" spans="1:37">
       <c r="A11" s="11" t="s">
@@ -2093,6 +2089,7 @@
       <c r="V11" s="20"/>
       <c r="W11" s="20"/>
       <c r="X11" s="20"/>
+      <c r="Y11" s="20"/>
     </row>
     <row r="12" spans="1:37">
       <c r="A12" s="11" t="s">
@@ -2166,6 +2163,9 @@
       </c>
       <c r="X12" s="20">
         <v>46267</v>
+      </c>
+      <c r="Y12" s="20">
+        <v>46268</v>
       </c>
       <c r="AK12" s="24" t="s">
         <v>252</v>
@@ -2305,6 +2305,7 @@
       <c r="V14" s="20"/>
       <c r="W14" s="20"/>
       <c r="X14" s="20"/>
+      <c r="Y14" s="20"/>
     </row>
     <row r="15" spans="1:37">
       <c r="A15" s="11" t="s">
@@ -3111,7 +3112,7 @@
       <c r="I33" s="21">
         <v>46363</v>
       </c>
-      <c r="J33" s="26">
+      <c r="J33" s="21">
         <v>46267</v>
       </c>
       <c r="K33" s="20"/>

</xml_diff>